<commit_message>
Link Kobo forms with monthly objectives
</commit_message>
<xml_diff>
--- a/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
+++ b/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rd3d88f90d5674c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R1477ff5ec1154e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Re619747b76fa4cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R8b5e7c4345ab4406"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R5a050ff3f0fa4308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R22086147a22c4102"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -893,12 +893,12 @@
         <x:v>valeur_cible</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>Valeur cible / objectif</x:v>
-      </x:c>
-      <x:c r="D17" s="24"/>
-      <x:c r="E17" s="24" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+        <x:v>Cible de reference optionnelle</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="str">
+        <x:v>Ne pas utiliser pour l'objectif mensuel officiel; utiliser le formulaire Objectifs mensuels.</x:v>
+      </x:c>
+      <x:c r="E17" s="24" t="str"/>
       <x:c r="F17" s="24"/>
       <x:c r="G17" s="24"/>
       <x:c r="H17" s="24"/>

</xml_diff>

<commit_message>
Use shared KPI IDs across Kobo forms
</commit_message>
<xml_diff>
--- a/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
+++ b/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R8b5e7c4345ab4406"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R5a050ff3f0fa4308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R22086147a22c4102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Re20d83b637354941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rd157404aa82c497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0c640d6ef4e44da6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -625,26 +625,28 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="23" t="str">
-        <x:v>text</x:v>
+        <x:v>select_one kpi_ids</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
         <x:v>id_kpi</x:v>
       </x:c>
       <x:c r="C5" s="24" t="str">
-        <x:v>ID KPI</x:v>
+        <x:v>ID KPI officiel</x:v>
       </x:c>
       <x:c r="D5" s="24" t="str">
-        <x:v>Ex. KPI-001 ou 01. Utiliser le meme ID dans le formulaire 2.</x:v>
+        <x:v>Choisir l'ID KPI officiel. Le meme ID doit etre repris dans Objectifs mensuels et Donnees de calcul.</x:v>
       </x:c>
       <x:c r="E5" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="F5" s="24"/>
       <x:c r="G5" s="24"/>
-      <x:c r="H5" s="24"/>
-      <x:c r="I5" s="24"/>
+      <x:c r="H5" s="24" t="str"/>
+      <x:c r="I5" s="24" t="str"/>
       <x:c r="J5" s="24"/>
-      <x:c r="K5" s="25"/>
+      <x:c r="K5" s="25" t="str">
+        <x:v>autocomplete</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="23" t="str">
@@ -2012,6 +2014,820 @@
       </x:c>
       <x:c r="C71" t="str">
         <x:v>Pole WFM (Workforce Management)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>KPI-001</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>KPI-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>KPI-002</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>KPI-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>KPI-003</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>KPI-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>KPI-004</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>KPI-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>KPI-005</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>KPI-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>KPI-006</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>KPI-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>KPI-007</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>KPI-007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>KPI-008</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>KPI-008</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>KPI-009</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>KPI-009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>KPI-010</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>KPI-010</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>KPI-011</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>KPI-011</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>KPI-012</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>KPI-012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>KPI-013</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>KPI-013</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>KPI-014</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>KPI-014</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>KPI-015</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>KPI-015</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>KPI-016</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>KPI-016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>KPI-017</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>KPI-017</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>KPI-018</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>KPI-018</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>KPI-019</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>KPI-019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>KPI-020</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>KPI-020</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>KPI-021</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>KPI-021</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>KPI-022</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>KPI-022</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>KPI-023</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>KPI-023</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>KPI-024</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>KPI-024</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>KPI-025</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>KPI-025</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>KPI-026</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>KPI-026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>KPI-027</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>KPI-027</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>KPI-028</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>KPI-028</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>KPI-029</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>KPI-029</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>KPI-030</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>KPI-030</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>KPI-031</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>KPI-031</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>KPI-032</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>KPI-032</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>KPI-033</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>KPI-033</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>KPI-034</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>KPI-034</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>KPI-035</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>KPI-035</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>KPI-036</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>KPI-036</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>KPI-037</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>KPI-037</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>KPI-038</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>KPI-038</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>KPI-039</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>KPI-039</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>KPI-040</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>KPI-040</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>KPI-041</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>KPI-041</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>KPI-042</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>KPI-042</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>KPI-043</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>KPI-043</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>KPI-044</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>KPI-044</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>KPI-045</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>KPI-045</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>KPI-046</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>KPI-046</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>KPI-047</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>KPI-047</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>KPI-048</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>KPI-048</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>KPI-049</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>KPI-049</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>KPI-050</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>KPI-050</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>KPI-051</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>KPI-051</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>KPI-052</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>KPI-052</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>KPI-053</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>KPI-053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>KPI-054</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>KPI-054</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>KPI-055</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>KPI-055</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>KPI-056</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>KPI-056</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>KPI-057</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>KPI-057</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>KPI-058</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>KPI-058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>KPI-059</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>KPI-059</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>KPI-060</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>KPI-060</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>KPI-061</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>KPI-061</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>KPI-062</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>KPI-062</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>KPI-063</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>KPI-063</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>KPI-064</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>KPI-064</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>KPI-065</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>KPI-065</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>KPI-066</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>KPI-066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>KPI-067</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>KPI-067</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B139" t="str">
+        <x:v>KPI-068</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>KPI-068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B140" t="str">
+        <x:v>KPI-069</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>KPI-069</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>KPI-070</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>KPI-070</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B142" t="str">
+        <x:v>KPI-071</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>KPI-071</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>KPI-072</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>KPI-072</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>KPI-073</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>KPI-073</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>KPI-074</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>KPI-074</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Expand Kobo KPI choices with labels
</commit_message>
<xml_diff>
--- a/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
+++ b/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026_corrige_pays_20260720.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Re20d83b637354941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rd157404aa82c497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0c640d6ef4e44da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rdbc9e66cf7484048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rdd9daff97c2948d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R25fb737f14b44590"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -634,7 +634,7 @@
         <x:v>ID KPI officiel</x:v>
       </x:c>
       <x:c r="D5" s="24" t="str">
-        <x:v>Choisir l'ID KPI officiel. Le meme ID doit etre repris dans Objectifs mensuels et Donnees de calcul.</x:v>
+        <x:v>Choisir l'ID KPI officiel. La liste affiche aussi l'intitule, la formule et la cible quand ils existent.</x:v>
       </x:c>
       <x:c r="E5" s="24" t="str">
         <x:v>yes</x:v>
@@ -2024,7 +2024,7 @@
         <x:v>KPI-001</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>KPI-001</x:v>
+        <x:v>KPI-001 - Chiffre d'affaires | Calcul: Volume produit x Prix unitaire HT | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -2035,7 +2035,7 @@
         <x:v>KPI-002</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>KPI-002</x:v>
+        <x:v>KPI-002 - Taux de maintenance préventive réalisés | Calcul: Nbre de maintenance préventive réalisé X 100) / Nbr de maintenance préve... | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -2046,7 +2046,7 @@
         <x:v>KPI-003</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>KPI-003</x:v>
+        <x:v>KPI-003 - Disponibilité / Accessibilité (système) | Calcul: Nombre de minutes de disponibilité des systèmes d’information X100) / To... | Cible: 98</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -2057,7 +2057,7 @@
         <x:v>KPI-004</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>KPI-004</x:v>
+        <x:v>KPI-004 - Transactions Bloquées (télécommunication) | Calcul: Nombre d’appels aboutissant à une tonalité d’occupation X100) / nombre t... | Cible: 98</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -2068,7 +2068,7 @@
         <x:v>KPI-005</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>KPI-005</x:v>
+        <x:v>KPI-005 - Taux de Disponibilité / Accessibilité (télécommunica... | Calcul: Nombre de minutes de disponibilité du commutateur X100) / Total des minu... | Cible: 98</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -2079,7 +2079,7 @@
         <x:v>KPI-006</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>KPI-006</x:v>
+        <x:v>KPI-006 - VOLUME IVR | Calcul: Nombre total de transaction éligible pour le service | Cible: 98</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -2090,7 +2090,7 @@
         <x:v>KPI-007</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>KPI-007</x:v>
+        <x:v>KPI-007 - TAUX DE FONCTIONNALITE DES SYSTEMES IVR | Calcul: Somme des temps d'indisponibilité X 100) / Temps total de disponibilité | Cible: 99</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -2101,7 +2101,7 @@
         <x:v>KPI-008</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>KPI-008</x:v>
+        <x:v>KPI-008 - Nombre d'incident de sécurité | Calcul: Nombre total d'incidents identifié sur le système informatique | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -2112,7 +2112,7 @@
         <x:v>KPI-009</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>KPI-009</x:v>
+        <x:v>KPI-009 - Taux de traitement dans les délais | Calcul: Nbre de ticket ouvert traités dans le délais(2880min)X100 / Nbre total d... | Cible: 89</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -2123,7 +2123,7 @@
         <x:v>KPI-010</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>KPI-010</x:v>
+        <x:v>KPI-010 - MTTR | Calcul: Moyenne de temps de traitement de tous les tickets sur la periode | Cible: 60</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -2134,7 +2134,7 @@
         <x:v>KPI-011</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>KPI-011</x:v>
+        <x:v>KPI-011 - Taux d'exactitude de réparation ou solution | Calcul: Volume total de tickets ouverts - Volume de tickets réouverts)X 100 / no... | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -2145,7 +2145,7 @@
         <x:v>KPI-012</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>KPI-012</x:v>
+        <x:v>KPI-012 - Tx Exact ECC | Calcul: Tx Exact ECC=Nb transactions sans ECC X 100/Nb transactions évaluées | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -2156,7 +2156,7 @@
         <x:v>KPI-013</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>KPI-013</x:v>
+        <x:v>KPI-013 - Tx Exact ECA | Calcul: Tx Exact ECA=Nb transactions sans ECA X 100/Nb transactions évaluées | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -2167,7 +2167,7 @@
         <x:v>KPI-014</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>KPI-014</x:v>
+        <x:v>KPI-014 - Tx Exact ECCo | Calcul: Tx Exact ECCo=Nb transactions sans ECCo X 100/Nb transactions évaluées | Cible: 99.5</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -2178,7 +2178,7 @@
         <x:v>KPI-015</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>KPI-015</x:v>
+        <x:v>KPI-015 - Tx Exact ENC | Calcul: Tx Exact ENC=Nb transactions sans ENC X 100/Nb transactions évaluées | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -2189,7 +2189,7 @@
         <x:v>KPI-016</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>KPI-016</x:v>
+        <x:v>KPI-016 - Tx défaut | Calcul: Tx défaut=Nb d'inconformité X 100/Nb transactions évaluées | Cible: 2</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -2200,7 +2200,7 @@
         <x:v>KPI-017</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>KPI-017</x:v>
+        <x:v>KPI-017 - Tx per de Esc | Calcul: Tx per de Esc= Pertinence de l’escalade = Nb d’escalades incorrectes / N... | Cible: 98</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -2211,7 +2211,7 @@
         <x:v>KPI-018</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>KPI-018</x:v>
+        <x:v>KPI-018 - VR | Calcul: VR=Echantillonnage représentatif sur le volume d’appels reçu. Calcul eff... | Cible: 600</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -2222,7 +2222,7 @@
         <x:v>KPI-019</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>KPI-019</x:v>
+        <x:v>KPI-019 - Taux de réussite Quiz FI | Calcul: Nombre d'apprenants ayant validé le quiz ÷ Nombre total d'apprenants aya... | Cible: 85</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -2233,7 +2233,7 @@
         <x:v>KPI-020</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>KPI-020</x:v>
+        <x:v>KPI-020 - Heures FI (Prévues vs Réalisées) | Calcul: Heures FI réalisées /Heures FI prévues)​ * 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -2244,7 +2244,7 @@
         <x:v>KPI-021</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>KPI-021</x:v>
+        <x:v>KPI-021 - Taux Présence Ateliers | Calcul: Nombre d'agents présents aux ateliers de formation ÷ Nombre d'agents con... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -2255,7 +2255,7 @@
         <x:v>KPI-022</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>KPI-022</x:v>
+        <x:v>KPI-022 - Taux de Présence au Coaching | Calcul: Nombre de séances de coaching réalisées ÷ Nombre de séances de coaching ... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -2266,7 +2266,7 @@
         <x:v>KPI-023</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>KPI-023</x:v>
+        <x:v>KPI-023 - Heures FC (Prévues vs Réalisées) | Calcul: Heures FC réalisées ÷ Heures FC prévues) × 100 | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -2277,7 +2277,7 @@
         <x:v>KPI-024</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>KPI-024</x:v>
+        <x:v>KPI-024 - Taux de Réussite Quiz FC | Calcul: Nombre d'agents ayant atteint ou dépassé le score minimum requis ÷ Nombr... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -2288,7 +2288,7 @@
         <x:v>KPI-025</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>KPI-025</x:v>
+        <x:v>KPI-025 - Score Quiz FC | Calcul: Somme des scores individuels obtenus aux quiz FC ÷ Nombre total d'agents... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -2299,7 +2299,7 @@
         <x:v>KPI-026</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>KPI-026</x:v>
+        <x:v>KPI-026 - Taux de complétion EDFLEX | Calcul: Nombre de parcours complétés ÷ Nombre de parcours assignés) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -2310,7 +2310,7 @@
         <x:v>KPI-027</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>KPI-027</x:v>
+        <x:v>KPI-027 - Qualité de la Formation CRCD — Intégration | Calcul: Nombre d'agents ayant réussi au quiz ÷ Nombre total d'agents évalués) × 100 | Cible: 85</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -2321,7 +2321,7 @@
         <x:v>KPI-028</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>KPI-028</x:v>
+        <x:v>KPI-028 - Qualité de la Formation CRCD — Continue | Calcul: Nombre d'agents ayant atteint le seuil ÷ Nombre total d'agents évalués) ... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -2332,7 +2332,7 @@
         <x:v>KPI-029</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>KPI-029</x:v>
+        <x:v>KPI-029 - Efficacité de la Formation | Calcul: Une enquête de satisfaction sur le déroulé de la formation | Cible: 80</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -2343,7 +2343,7 @@
         <x:v>KPI-030</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>KPI-030</x:v>
+        <x:v>KPI-030 - Efficacité du Formateur | Calcul: feedbacks à chaud ( enquête de satisfaction) | Cible: 80</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -2354,7 +2354,7 @@
         <x:v>KPI-031</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>KPI-031</x:v>
+        <x:v>KPI-031 - Taux de Formation Réalisée | Calcul: Nombre de formation réalisée / Nombre de formation prévue) * 100 | Cible: 60</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -2365,7 +2365,7 @@
         <x:v>KPI-032</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>KPI-032</x:v>
+        <x:v>KPI-032 - FOLLOWERS LINKEDIN | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -2376,7 +2376,7 @@
         <x:v>KPI-033</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>KPI-033</x:v>
+        <x:v>KPI-033 - FOLLOWERS FACEBOOK | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -2387,7 +2387,7 @@
         <x:v>KPI-034</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>KPI-034</x:v>
+        <x:v>KPI-034 - FOLLOWERS INSTAGRAM | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -2398,7 +2398,7 @@
         <x:v>KPI-035</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>KPI-035</x:v>
+        <x:v>KPI-035 - FOLLOWERS SUR X (Twitter) | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -2409,7 +2409,7 @@
         <x:v>KPI-036</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>KPI-036</x:v>
+        <x:v>KPI-036 - IMPRESSION (LINKEDIN) | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -2420,7 +2420,7 @@
         <x:v>KPI-037</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>KPI-037</x:v>
+        <x:v>KPI-037 - PORTEE (FACEBOOK) | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -2431,7 +2431,7 @@
         <x:v>KPI-038</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>KPI-038</x:v>
+        <x:v>KPI-038 - PORTEE (INSTAGRAM) | Calcul: NA | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -2442,7 +2442,7 @@
         <x:v>KPI-039</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>KPI-039</x:v>
+        <x:v>KPI-039 - TAUX D'ENGAGEMENT | Calcul: INTERACTIONS/IMPRESSIONS) *100 | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -2453,7 +2453,7 @@
         <x:v>KPI-040</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>KPI-040</x:v>
+        <x:v>KPI-040 - TAUX D'ENGAGEMENT FACEBOOK | Calcul: INTERACTIONS/PORTEE) * 100 | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -2464,7 +2464,7 @@
         <x:v>KPI-041</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>KPI-041</x:v>
+        <x:v>KPI-041 - TAUX D'ENGAGEMENT INSTAGRAM | Calcul: INTERACTIONS/PORTEE) *100 | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -2475,7 +2475,7 @@
         <x:v>KPI-042</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>KPI-042</x:v>
+        <x:v>KPI-042 - Masse Salariale | Calcul: Total des charges RH sur le total du Chiffre d'affaires | Cible: 35</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -2486,7 +2486,7 @@
         <x:v>KPI-043</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>KPI-043</x:v>
+        <x:v>KPI-043 - Résultat Avant Impôt | Calcul: Chiffre d'affaires - toutes charges) / Chiffre d'affaires | Cible: 15</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -2497,7 +2497,7 @@
         <x:v>KPI-044</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>KPI-044</x:v>
+        <x:v>KPI-044 - Taux de transformation digital | Calcul: Somme (%projet) / Nombre de projets | Cible: 70</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -2508,7 +2508,7 @@
         <x:v>KPI-045</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>KPI-045</x:v>
+        <x:v>KPI-045 - Taux de recouvrement | Calcul: Somme des encaissements sur la période / Somme des créances exigibles su... | Cible: 75</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -2519,7 +2519,7 @@
         <x:v>KPI-046</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>KPI-046</x:v>
+        <x:v>KPI-046 - Créances clients | Calcul: Somme des factures émises échues sur une période donnée | Cible: 1</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -2530,7 +2530,7 @@
         <x:v>KPI-047</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>KPI-047</x:v>
+        <x:v>KPI-047 - Encours Clients | Calcul: Somme des créances clients (Factures échues et non échues) + Commandes e... | Cible: 1</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -2541,7 +2541,7 @@
         <x:v>KPI-048</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>KPI-048</x:v>
+        <x:v>KPI-048 - Balance Âgée | Calcul: Date du jour - date d'échéance de la facture | Cible: 25</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -2552,7 +2552,7 @@
         <x:v>KPI-049</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>KPI-049</x:v>
+        <x:v>KPI-049 - DSO (Days Sales Outstanding) | Calcul: Créances clients / Chiffre d’affaires TTC sur la période) × Nombre de jo... | Cible: 45</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -2563,7 +2563,7 @@
         <x:v>KPI-050</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>KPI-050</x:v>
+        <x:v>KPI-050 - Point des Encaissements | Calcul: Somme réelle des encaissements sur une période donnée (virements, chèque... | Cible: 1</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -2574,7 +2574,7 @@
         <x:v>KPI-051</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>KPI-051</x:v>
+        <x:v>KPI-051 - Créances Irrécouvrables | Calcul: Créances douteuses / CA total). | Cible: 5</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -2585,7 +2585,7 @@
         <x:v>KPI-052</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>KPI-052</x:v>
+        <x:v>KPI-052 - ADHERENCE HEURE | Calcul: Heures réalisées (temps total de présence - temps de déjeuner) /heures p... | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -2596,7 +2596,7 @@
         <x:v>KPI-053</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>KPI-053</x:v>
+        <x:v>KPI-053 - TAUX D'OCCUPATION | Calcul: Traitement + attente ) /( Traitement + attente + post appel ) )* 100 | Cible: 75</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -2607,7 +2607,7 @@
         <x:v>KPI-054</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>KPI-054</x:v>
+        <x:v>KPI-054 - ADHERENCE PLANNING | Calcul: ETP (EFFECTIF TOTAL PLANIFIES) / BESOIN ) )* 100 | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -2618,7 +2618,7 @@
         <x:v>KPI-055</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>KPI-055</x:v>
+        <x:v>KPI-055 - QUALITE DE PREVISION | Calcul: RECUS / PREVUS | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -2629,7 +2629,7 @@
         <x:v>KPI-056</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>KPI-056</x:v>
+        <x:v>KPI-056 - EFFICACITE | Calcul: TRAITES/RECUS | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -2640,7 +2640,7 @@
         <x:v>KPI-057</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>KPI-057</x:v>
+        <x:v>KPI-057 - Volume total des achats | Calcul: Somme des montants des bons de commande et bons d'achat émis sur la période | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -2651,7 +2651,7 @@
         <x:v>KPI-058</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>KPI-058</x:v>
+        <x:v>KPI-058 - Taux de conformité des bons de commande | Calcul: Nombre de bons de commande conformes / Nombre total de bons de commande)... | Cible: 95</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -2662,7 +2662,7 @@
         <x:v>KPI-059</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>KPI-059</x:v>
+        <x:v>KPI-059 - Taux de non-conformité des produits | Calcul: Nombre de produits retournés ou non conformes / Total des produits achet... | Cible: 1</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -2673,7 +2673,7 @@
         <x:v>KPI-060</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>KPI-060</x:v>
+        <x:v>KPI-060 - Délai moyen d'approvisionnement | Calcul: Somme des délais individuels d'approvisionnement / Nombre de demandes tr... | Cible: a definir</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -2684,7 +2684,7 @@
         <x:v>KPI-061</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>KPI-061</x:v>
+        <x:v>KPI-061 - Taux de service client | Calcul: Nombre de demandes satisfaites / Nombre total de demandes exprimées) × 100 | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -2695,7 +2695,7 @@
         <x:v>KPI-062</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>KPI-062</x:v>
+        <x:v>KPI-062 - Taux de disponibilité du stock critique | Calcul: Nombre d'articles critiques disponibles / Nombre total d'articles critiq... | Cible: 90</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -2706,7 +2706,7 @@
         <x:v>KPI-063</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>KPI-063</x:v>
+        <x:v>KPI-063 - OOS | Calcul: TRO OOS (%) = Objectif (%) /Réalisé(%) | Cible: 19.7</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -2717,7 +2717,7 @@
         <x:v>KPI-064</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>KPI-064</x:v>
+        <x:v>KPI-064 - DTR (Direct To Retail) | Calcul: TRO DTR (%) = (Réalisé DTR / Objectif DTR) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -2728,7 +2728,7 @@
         <x:v>KPI-065</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>KPI-065</x:v>
+        <x:v>KPI-065 - DTC (Direct To Consumer) | Calcul: TRO DTC (%) = (Réalisé DTC / Objectif DTC) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -2739,7 +2739,7 @@
         <x:v>KPI-066</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>KPI-066</x:v>
+        <x:v>KPI-066 - ADU (Active Data Users) | Calcul: TRO ADU (%) = (ADU Réalisé / ADU Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -2750,7 +2750,7 @@
         <x:v>KPI-067</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>KPI-067</x:v>
+        <x:v>KPI-067 - MAU (MoMo Active Users) | Calcul: TRO MAU (%) = (MAU Réalisé / MAU Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -2761,7 +2761,7 @@
         <x:v>KPI-068</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>KPI-068</x:v>
+        <x:v>KPI-068 - FTTH (Fiber To The Home) | Calcul: TRO FTTH (%) = (FTTH Réalisé / FTTH Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -2772,7 +2772,7 @@
         <x:v>KPI-069</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>KPI-069</x:v>
+        <x:v>KPI-069 - FWA (Fixed Wireless Access) | Calcul: TRO FWA (%) = (FWA Réalisé / FWA Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -2783,7 +2783,7 @@
         <x:v>KPI-070</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>KPI-070</x:v>
+        <x:v>KPI-070 - Services at Touch Point (SATP) | Calcul: SATP(%) = (NPS AGENT + NPS AGENCE)/2 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -2794,7 +2794,7 @@
         <x:v>KPI-071</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>KPI-071</x:v>
+        <x:v>KPI-071 - Recrutement Commerciaux (MRE) | Calcul: TRO = (Réalisé / Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -2805,7 +2805,7 @@
         <x:v>KPI-072</x:v>
       </x:c>
       <x:c r="C143" t="str">
-        <x:v>KPI-072</x:v>
+        <x:v>KPI-072 - Performance MRE | Calcul: TRO = (Réalisé / Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -2816,7 +2816,7 @@
         <x:v>KPI-073</x:v>
       </x:c>
       <x:c r="C144" t="str">
-        <x:v>KPI-073</x:v>
+        <x:v>KPI-073 - Recrutement TDR | Calcul: TRO = (Réalisé / Objectif) × 100 | Cible: 100</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -2827,7 +2827,1393 @@
         <x:v>KPI-074</x:v>
       </x:c>
       <x:c r="C145" t="str">
-        <x:v>KPI-074</x:v>
+        <x:v>KPI-074 - Performance TDR | Calcul: TRO = (Réalisé / Objectif) × 100 | Cible: 100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>KPI-075</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>KPI-075 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>KPI-076</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>KPI-076 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>KPI-077</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>KPI-077 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>KPI-078</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>KPI-078 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>KPI-079</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>KPI-079 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>KPI-080</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>KPI-080 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>KPI-081</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>KPI-081 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>KPI-082</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>KPI-082 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>KPI-083</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>KPI-083 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>KPI-084</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>KPI-084 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>KPI-085</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>KPI-085 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>KPI-086</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>KPI-086 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>KPI-087</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>KPI-087 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>KPI-088</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>KPI-088 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B160" t="str">
+        <x:v>KPI-089</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>KPI-089 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B161" t="str">
+        <x:v>KPI-090</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>KPI-090 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B162" t="str">
+        <x:v>KPI-091</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>KPI-091 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B163" t="str">
+        <x:v>KPI-092</x:v>
+      </x:c>
+      <x:c r="C163" t="str">
+        <x:v>KPI-092 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>KPI-093</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>KPI-093 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B165" t="str">
+        <x:v>KPI-094</x:v>
+      </x:c>
+      <x:c r="C165" t="str">
+        <x:v>KPI-094 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B166" t="str">
+        <x:v>KPI-095</x:v>
+      </x:c>
+      <x:c r="C166" t="str">
+        <x:v>KPI-095 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B167" t="str">
+        <x:v>KPI-096</x:v>
+      </x:c>
+      <x:c r="C167" t="str">
+        <x:v>KPI-096 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B168" t="str">
+        <x:v>KPI-097</x:v>
+      </x:c>
+      <x:c r="C168" t="str">
+        <x:v>KPI-097 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B169" t="str">
+        <x:v>KPI-098</x:v>
+      </x:c>
+      <x:c r="C169" t="str">
+        <x:v>KPI-098 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B170" t="str">
+        <x:v>KPI-099</x:v>
+      </x:c>
+      <x:c r="C170" t="str">
+        <x:v>KPI-099 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>KPI-100</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>KPI-100 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B172" t="str">
+        <x:v>KPI-101</x:v>
+      </x:c>
+      <x:c r="C172" t="str">
+        <x:v>KPI-101 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B173" t="str">
+        <x:v>KPI-102</x:v>
+      </x:c>
+      <x:c r="C173" t="str">
+        <x:v>KPI-102 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B174" t="str">
+        <x:v>KPI-103</x:v>
+      </x:c>
+      <x:c r="C174" t="str">
+        <x:v>KPI-103 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B175" t="str">
+        <x:v>KPI-104</x:v>
+      </x:c>
+      <x:c r="C175" t="str">
+        <x:v>KPI-104 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B176" t="str">
+        <x:v>KPI-105</x:v>
+      </x:c>
+      <x:c r="C176" t="str">
+        <x:v>KPI-105 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B177" t="str">
+        <x:v>KPI-106</x:v>
+      </x:c>
+      <x:c r="C177" t="str">
+        <x:v>KPI-106 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B178" t="str">
+        <x:v>KPI-107</x:v>
+      </x:c>
+      <x:c r="C178" t="str">
+        <x:v>KPI-107 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B179" t="str">
+        <x:v>KPI-108</x:v>
+      </x:c>
+      <x:c r="C179" t="str">
+        <x:v>KPI-108 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B180" t="str">
+        <x:v>KPI-109</x:v>
+      </x:c>
+      <x:c r="C180" t="str">
+        <x:v>KPI-109 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B181" t="str">
+        <x:v>KPI-110</x:v>
+      </x:c>
+      <x:c r="C181" t="str">
+        <x:v>KPI-110 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B182" t="str">
+        <x:v>KPI-111</x:v>
+      </x:c>
+      <x:c r="C182" t="str">
+        <x:v>KPI-111 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B183" t="str">
+        <x:v>KPI-112</x:v>
+      </x:c>
+      <x:c r="C183" t="str">
+        <x:v>KPI-112 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B184" t="str">
+        <x:v>KPI-113</x:v>
+      </x:c>
+      <x:c r="C184" t="str">
+        <x:v>KPI-113 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B185" t="str">
+        <x:v>KPI-114</x:v>
+      </x:c>
+      <x:c r="C185" t="str">
+        <x:v>KPI-114 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B186" t="str">
+        <x:v>KPI-115</x:v>
+      </x:c>
+      <x:c r="C186" t="str">
+        <x:v>KPI-115 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B187" t="str">
+        <x:v>KPI-116</x:v>
+      </x:c>
+      <x:c r="C187" t="str">
+        <x:v>KPI-116 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B188" t="str">
+        <x:v>KPI-117</x:v>
+      </x:c>
+      <x:c r="C188" t="str">
+        <x:v>KPI-117 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B189" t="str">
+        <x:v>KPI-118</x:v>
+      </x:c>
+      <x:c r="C189" t="str">
+        <x:v>KPI-118 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B190" t="str">
+        <x:v>KPI-119</x:v>
+      </x:c>
+      <x:c r="C190" t="str">
+        <x:v>KPI-119 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B191" t="str">
+        <x:v>KPI-120</x:v>
+      </x:c>
+      <x:c r="C191" t="str">
+        <x:v>KPI-120 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B192" t="str">
+        <x:v>KPI-121</x:v>
+      </x:c>
+      <x:c r="C192" t="str">
+        <x:v>KPI-121 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B193" t="str">
+        <x:v>KPI-122</x:v>
+      </x:c>
+      <x:c r="C193" t="str">
+        <x:v>KPI-122 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B194" t="str">
+        <x:v>KPI-123</x:v>
+      </x:c>
+      <x:c r="C194" t="str">
+        <x:v>KPI-123 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B195" t="str">
+        <x:v>KPI-124</x:v>
+      </x:c>
+      <x:c r="C195" t="str">
+        <x:v>KPI-124 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B196" t="str">
+        <x:v>KPI-125</x:v>
+      </x:c>
+      <x:c r="C196" t="str">
+        <x:v>KPI-125 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B197" t="str">
+        <x:v>KPI-126</x:v>
+      </x:c>
+      <x:c r="C197" t="str">
+        <x:v>KPI-126 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B198" t="str">
+        <x:v>KPI-127</x:v>
+      </x:c>
+      <x:c r="C198" t="str">
+        <x:v>KPI-127 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B199" t="str">
+        <x:v>KPI-128</x:v>
+      </x:c>
+      <x:c r="C199" t="str">
+        <x:v>KPI-128 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B200" t="str">
+        <x:v>KPI-129</x:v>
+      </x:c>
+      <x:c r="C200" t="str">
+        <x:v>KPI-129 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B201" t="str">
+        <x:v>KPI-130</x:v>
+      </x:c>
+      <x:c r="C201" t="str">
+        <x:v>KPI-130 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B202" t="str">
+        <x:v>KPI-131</x:v>
+      </x:c>
+      <x:c r="C202" t="str">
+        <x:v>KPI-131 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B203" t="str">
+        <x:v>KPI-132</x:v>
+      </x:c>
+      <x:c r="C203" t="str">
+        <x:v>KPI-132 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B204" t="str">
+        <x:v>KPI-133</x:v>
+      </x:c>
+      <x:c r="C204" t="str">
+        <x:v>KPI-133 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B205" t="str">
+        <x:v>KPI-134</x:v>
+      </x:c>
+      <x:c r="C205" t="str">
+        <x:v>KPI-134 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B206" t="str">
+        <x:v>KPI-135</x:v>
+      </x:c>
+      <x:c r="C206" t="str">
+        <x:v>KPI-135 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B207" t="str">
+        <x:v>KPI-136</x:v>
+      </x:c>
+      <x:c r="C207" t="str">
+        <x:v>KPI-136 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B208" t="str">
+        <x:v>KPI-137</x:v>
+      </x:c>
+      <x:c r="C208" t="str">
+        <x:v>KPI-137 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B209" t="str">
+        <x:v>KPI-138</x:v>
+      </x:c>
+      <x:c r="C209" t="str">
+        <x:v>KPI-138 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="A210" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B210" t="str">
+        <x:v>KPI-139</x:v>
+      </x:c>
+      <x:c r="C210" t="str">
+        <x:v>KPI-139 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211">
+      <x:c r="A211" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B211" t="str">
+        <x:v>KPI-140</x:v>
+      </x:c>
+      <x:c r="C211" t="str">
+        <x:v>KPI-140 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="A212" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B212" t="str">
+        <x:v>KPI-141</x:v>
+      </x:c>
+      <x:c r="C212" t="str">
+        <x:v>KPI-141 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B213" t="str">
+        <x:v>KPI-142</x:v>
+      </x:c>
+      <x:c r="C213" t="str">
+        <x:v>KPI-142 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="A214" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B214" t="str">
+        <x:v>KPI-143</x:v>
+      </x:c>
+      <x:c r="C214" t="str">
+        <x:v>KPI-143 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="A215" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B215" t="str">
+        <x:v>KPI-144</x:v>
+      </x:c>
+      <x:c r="C215" t="str">
+        <x:v>KPI-144 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="A216" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B216" t="str">
+        <x:v>KPI-145</x:v>
+      </x:c>
+      <x:c r="C216" t="str">
+        <x:v>KPI-145 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="A217" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B217" t="str">
+        <x:v>KPI-146</x:v>
+      </x:c>
+      <x:c r="C217" t="str">
+        <x:v>KPI-146 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="A218" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B218" t="str">
+        <x:v>KPI-147</x:v>
+      </x:c>
+      <x:c r="C218" t="str">
+        <x:v>KPI-147 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="A219" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B219" t="str">
+        <x:v>KPI-148</x:v>
+      </x:c>
+      <x:c r="C219" t="str">
+        <x:v>KPI-148 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="A220" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B220" t="str">
+        <x:v>KPI-149</x:v>
+      </x:c>
+      <x:c r="C220" t="str">
+        <x:v>KPI-149 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221">
+      <x:c r="A221" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B221" t="str">
+        <x:v>KPI-150</x:v>
+      </x:c>
+      <x:c r="C221" t="str">
+        <x:v>KPI-150 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B222" t="str">
+        <x:v>KPI-151</x:v>
+      </x:c>
+      <x:c r="C222" t="str">
+        <x:v>KPI-151 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B223" t="str">
+        <x:v>KPI-152</x:v>
+      </x:c>
+      <x:c r="C223" t="str">
+        <x:v>KPI-152 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B224" t="str">
+        <x:v>KPI-153</x:v>
+      </x:c>
+      <x:c r="C224" t="str">
+        <x:v>KPI-153 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B225" t="str">
+        <x:v>KPI-154</x:v>
+      </x:c>
+      <x:c r="C225" t="str">
+        <x:v>KPI-154 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B226" t="str">
+        <x:v>KPI-155</x:v>
+      </x:c>
+      <x:c r="C226" t="str">
+        <x:v>KPI-155 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B227" t="str">
+        <x:v>KPI-156</x:v>
+      </x:c>
+      <x:c r="C227" t="str">
+        <x:v>KPI-156 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B228" t="str">
+        <x:v>KPI-157</x:v>
+      </x:c>
+      <x:c r="C228" t="str">
+        <x:v>KPI-157 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B229" t="str">
+        <x:v>KPI-158</x:v>
+      </x:c>
+      <x:c r="C229" t="str">
+        <x:v>KPI-158 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B230" t="str">
+        <x:v>KPI-159</x:v>
+      </x:c>
+      <x:c r="C230" t="str">
+        <x:v>KPI-159 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B231" t="str">
+        <x:v>KPI-160</x:v>
+      </x:c>
+      <x:c r="C231" t="str">
+        <x:v>KPI-160 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B232" t="str">
+        <x:v>KPI-161</x:v>
+      </x:c>
+      <x:c r="C232" t="str">
+        <x:v>KPI-161 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B233" t="str">
+        <x:v>KPI-162</x:v>
+      </x:c>
+      <x:c r="C233" t="str">
+        <x:v>KPI-162 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B234" t="str">
+        <x:v>KPI-163</x:v>
+      </x:c>
+      <x:c r="C234" t="str">
+        <x:v>KPI-163 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B235" t="str">
+        <x:v>KPI-164</x:v>
+      </x:c>
+      <x:c r="C235" t="str">
+        <x:v>KPI-164 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B236" t="str">
+        <x:v>KPI-165</x:v>
+      </x:c>
+      <x:c r="C236" t="str">
+        <x:v>KPI-165 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B237" t="str">
+        <x:v>KPI-166</x:v>
+      </x:c>
+      <x:c r="C237" t="str">
+        <x:v>KPI-166 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238">
+      <x:c r="A238" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B238" t="str">
+        <x:v>KPI-167</x:v>
+      </x:c>
+      <x:c r="C238" t="str">
+        <x:v>KPI-167 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239">
+      <x:c r="A239" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B239" t="str">
+        <x:v>KPI-168</x:v>
+      </x:c>
+      <x:c r="C239" t="str">
+        <x:v>KPI-168 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="A240" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B240" t="str">
+        <x:v>KPI-169</x:v>
+      </x:c>
+      <x:c r="C240" t="str">
+        <x:v>KPI-169 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241">
+      <x:c r="A241" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B241" t="str">
+        <x:v>KPI-170</x:v>
+      </x:c>
+      <x:c r="C241" t="str">
+        <x:v>KPI-170 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242">
+      <x:c r="A242" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B242" t="str">
+        <x:v>KPI-171</x:v>
+      </x:c>
+      <x:c r="C242" t="str">
+        <x:v>KPI-171 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243">
+      <x:c r="A243" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B243" t="str">
+        <x:v>KPI-172</x:v>
+      </x:c>
+      <x:c r="C243" t="str">
+        <x:v>KPI-172 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244">
+      <x:c r="A244" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B244" t="str">
+        <x:v>KPI-173</x:v>
+      </x:c>
+      <x:c r="C244" t="str">
+        <x:v>KPI-173 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245">
+      <x:c r="A245" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B245" t="str">
+        <x:v>KPI-174</x:v>
+      </x:c>
+      <x:c r="C245" t="str">
+        <x:v>KPI-174 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246">
+      <x:c r="A246" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B246" t="str">
+        <x:v>KPI-175</x:v>
+      </x:c>
+      <x:c r="C246" t="str">
+        <x:v>KPI-175 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B247" t="str">
+        <x:v>KPI-176</x:v>
+      </x:c>
+      <x:c r="C247" t="str">
+        <x:v>KPI-176 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="A248" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B248" t="str">
+        <x:v>KPI-177</x:v>
+      </x:c>
+      <x:c r="C248" t="str">
+        <x:v>KPI-177 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="A249" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B249" t="str">
+        <x:v>KPI-178</x:v>
+      </x:c>
+      <x:c r="C249" t="str">
+        <x:v>KPI-178 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="A250" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B250" t="str">
+        <x:v>KPI-179</x:v>
+      </x:c>
+      <x:c r="C250" t="str">
+        <x:v>KPI-179 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251">
+      <x:c r="A251" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B251" t="str">
+        <x:v>KPI-180</x:v>
+      </x:c>
+      <x:c r="C251" t="str">
+        <x:v>KPI-180 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B252" t="str">
+        <x:v>KPI-181</x:v>
+      </x:c>
+      <x:c r="C252" t="str">
+        <x:v>KPI-181 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253">
+      <x:c r="A253" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B253" t="str">
+        <x:v>KPI-182</x:v>
+      </x:c>
+      <x:c r="C253" t="str">
+        <x:v>KPI-182 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254">
+      <x:c r="A254" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B254" t="str">
+        <x:v>KPI-183</x:v>
+      </x:c>
+      <x:c r="C254" t="str">
+        <x:v>KPI-183 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255">
+      <x:c r="A255" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B255" t="str">
+        <x:v>KPI-184</x:v>
+      </x:c>
+      <x:c r="C255" t="str">
+        <x:v>KPI-184 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B256" t="str">
+        <x:v>KPI-185</x:v>
+      </x:c>
+      <x:c r="C256" t="str">
+        <x:v>KPI-185 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B257" t="str">
+        <x:v>KPI-186</x:v>
+      </x:c>
+      <x:c r="C257" t="str">
+        <x:v>KPI-186 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B258" t="str">
+        <x:v>KPI-187</x:v>
+      </x:c>
+      <x:c r="C258" t="str">
+        <x:v>KPI-187 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B259" t="str">
+        <x:v>KPI-188</x:v>
+      </x:c>
+      <x:c r="C259" t="str">
+        <x:v>KPI-188 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="A260" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B260" t="str">
+        <x:v>KPI-189</x:v>
+      </x:c>
+      <x:c r="C260" t="str">
+        <x:v>KPI-189 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="A261" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B261" t="str">
+        <x:v>KPI-190</x:v>
+      </x:c>
+      <x:c r="C261" t="str">
+        <x:v>KPI-190 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B262" t="str">
+        <x:v>KPI-191</x:v>
+      </x:c>
+      <x:c r="C262" t="str">
+        <x:v>KPI-191 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B263" t="str">
+        <x:v>KPI-192</x:v>
+      </x:c>
+      <x:c r="C263" t="str">
+        <x:v>KPI-192 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B264" t="str">
+        <x:v>KPI-193</x:v>
+      </x:c>
+      <x:c r="C264" t="str">
+        <x:v>KPI-193 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B265" t="str">
+        <x:v>KPI-194</x:v>
+      </x:c>
+      <x:c r="C265" t="str">
+        <x:v>KPI-194 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B266" t="str">
+        <x:v>KPI-195</x:v>
+      </x:c>
+      <x:c r="C266" t="str">
+        <x:v>KPI-195 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B267" t="str">
+        <x:v>KPI-196</x:v>
+      </x:c>
+      <x:c r="C267" t="str">
+        <x:v>KPI-196 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="A268" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B268" t="str">
+        <x:v>KPI-197</x:v>
+      </x:c>
+      <x:c r="C268" t="str">
+        <x:v>KPI-197 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B269" t="str">
+        <x:v>KPI-198</x:v>
+      </x:c>
+      <x:c r="C269" t="str">
+        <x:v>KPI-198 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="A270" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B270" t="str">
+        <x:v>KPI-199</x:v>
+      </x:c>
+      <x:c r="C270" t="str">
+        <x:v>KPI-199 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271">
+      <x:c r="A271" t="str">
+        <x:v>kpi_ids</x:v>
+      </x:c>
+      <x:c r="B271" t="str">
+        <x:v>KPI-200</x:v>
+      </x:c>
+      <x:c r="C271" t="str">
+        <x:v>KPI-200 - Reserve nouveau KPI | A declarer dans le Formulaire 1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>